<commit_message>
installation: two separates files for linux (install_linux.sh) and for windows (install_win.bat)
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -523,7 +523,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-24 03:27</t>
+          <t>2026-09-24 03:55</t>
         </is>
       </c>
       <c r="K2" t="inlineStr"/>
@@ -570,7 +570,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-24 03:27</t>
+          <t>2026-09-24 03:55</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
@@ -617,7 +617,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-24 03:27</t>
+          <t>2026-09-24 03:55</t>
         </is>
       </c>
       <c r="K4" t="inlineStr"/>

</xml_diff>